<commit_message>
Uploading file via API
</commit_message>
<xml_diff>
--- a/file-upload/Book1.xlsx
+++ b/file-upload/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya.yerramsetti\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBEE62AD-F24E-41B4-BC68-476B6BC5D244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F5FADE-A4C2-499B-B25B-537EC973605C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{77040213-5556-49A9-A916-37947BFECD2F}"/>
   </bookViews>
@@ -36,12 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="1">
   <si>
-    <t>check c</t>
-  </si>
-  <si>
-    <t>dfsf</t>
+    <t>me</t>
   </si>
 </sst>
 </file>
@@ -421,7 +418,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>